<commit_message>
BWI sync — 2026-07-06 12:56 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Argentina.xlsx
+++ b/BWI/bestwine_output/bestwine_Argentina.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA326"/>
+  <dimension ref="A1:AA328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -31951,6 +31951,216 @@
       <c r="Z326" s="2" t="inlineStr"/>
       <c r="AA326" s="2" t="inlineStr"/>
     </row>
+    <row r="327">
+      <c r="A327" s="2" t="inlineStr">
+        <is>
+          <t>ñuke Mapu S.r.l.</t>
+        </is>
+      </c>
+      <c r="B327" s="2" t="inlineStr">
+        <is>
+          <t>ñuke Mapu S.r.l.</t>
+        </is>
+      </c>
+      <c r="C327" s="2" t="inlineStr">
+        <is>
+          <t>122030</t>
+        </is>
+      </c>
+      <c r="D327" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E327" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F327" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous City of Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G327" s="2" t="inlineStr">
+        <is>
+          <t>3968 Avenida Pavón</t>
+        </is>
+      </c>
+      <c r="H327" s="2" t="inlineStr">
+        <is>
+          <t>C1253</t>
+        </is>
+      </c>
+      <c r="I327" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nukemapuvinos.com</t>
+        </is>
+      </c>
+      <c r="J327" s="2" t="inlineStr"/>
+      <c r="K327" s="2" t="inlineStr"/>
+      <c r="L327" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M327" s="2" t="inlineStr"/>
+      <c r="N327" s="2" t="inlineStr">
+        <is>
+          <t>nukemapu.ig@gmail.com</t>
+        </is>
+      </c>
+      <c r="O327" s="2" t="inlineStr">
+        <is>
+          <t>+54 11 4924-1087</t>
+        </is>
+      </c>
+      <c r="P327" s="2" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="Q327" s="2" t="inlineStr">
+        <is>
+          <t>30-70942499-4</t>
+        </is>
+      </c>
+      <c r="R327" s="2" t="inlineStr"/>
+      <c r="S327" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/nukemapudistribuidora/</t>
+        </is>
+      </c>
+      <c r="T327" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nukemapuvinos/</t>
+        </is>
+      </c>
+      <c r="U327" s="2" t="inlineStr"/>
+      <c r="V327" s="2" t="inlineStr"/>
+      <c r="W327" s="2" t="inlineStr">
+        <is>
+          <t>Anyelen Piragine</t>
+        </is>
+      </c>
+      <c r="X327" s="2" t="inlineStr">
+        <is>
+          <t>Administration Manager</t>
+        </is>
+      </c>
+      <c r="Y327" s="2" t="inlineStr"/>
+      <c r="Z327" s="2" t="inlineStr"/>
+      <c r="AA327" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/anyelen-piragine-23b5b9b1/</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="2" t="inlineStr">
+        <is>
+          <t>ñuke Mapu S.r.l.</t>
+        </is>
+      </c>
+      <c r="B328" s="2" t="inlineStr">
+        <is>
+          <t>ñuke Mapu S.r.l.</t>
+        </is>
+      </c>
+      <c r="C328" s="2" t="inlineStr">
+        <is>
+          <t>122030</t>
+        </is>
+      </c>
+      <c r="D328" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E328" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F328" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous City of Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G328" s="2" t="inlineStr">
+        <is>
+          <t>3968 Avenida Pavón</t>
+        </is>
+      </c>
+      <c r="H328" s="2" t="inlineStr">
+        <is>
+          <t>C1253</t>
+        </is>
+      </c>
+      <c r="I328" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nukemapuvinos.com</t>
+        </is>
+      </c>
+      <c r="J328" s="2" t="inlineStr"/>
+      <c r="K328" s="2" t="inlineStr"/>
+      <c r="L328" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M328" s="2" t="inlineStr"/>
+      <c r="N328" s="2" t="inlineStr">
+        <is>
+          <t>nukemapu.ig@gmail.com</t>
+        </is>
+      </c>
+      <c r="O328" s="2" t="inlineStr">
+        <is>
+          <t>+54 11 4924-1087</t>
+        </is>
+      </c>
+      <c r="P328" s="2" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="Q328" s="2" t="inlineStr">
+        <is>
+          <t>30-70942499-4</t>
+        </is>
+      </c>
+      <c r="R328" s="2" t="inlineStr"/>
+      <c r="S328" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/nukemapudistribuidora/</t>
+        </is>
+      </c>
+      <c r="T328" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nukemapuvinos/</t>
+        </is>
+      </c>
+      <c r="U328" s="2" t="inlineStr"/>
+      <c r="V328" s="2" t="inlineStr"/>
+      <c r="W328" s="2" t="inlineStr">
+        <is>
+          <t>Ignacio Hernandez</t>
+        </is>
+      </c>
+      <c r="X328" s="2" t="inlineStr">
+        <is>
+          <t>Administrative Assistant</t>
+        </is>
+      </c>
+      <c r="Y328" s="2" t="inlineStr"/>
+      <c r="Z328" s="2" t="inlineStr"/>
+      <c r="AA328" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ignacio-hernandez-9152b9145/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BWI sync — 2026-07-13 12:16 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Argentina.xlsx
+++ b/BWI/bestwine_output/bestwine_Argentina.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA328"/>
+  <dimension ref="A1:AA329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -32161,6 +32161,95 @@
         </is>
       </c>
     </row>
+    <row r="329">
+      <c r="A329" s="2" t="inlineStr">
+        <is>
+          <t>Club Segunda Copa</t>
+        </is>
+      </c>
+      <c r="B329" s="2" t="inlineStr">
+        <is>
+          <t>Club Segunda Copa</t>
+        </is>
+      </c>
+      <c r="C329" s="2" t="inlineStr">
+        <is>
+          <t>143</t>
+        </is>
+      </c>
+      <c r="D329" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E329" s="2" t="inlineStr">
+        <is>
+          <t>Martínez</t>
+        </is>
+      </c>
+      <c r="F329" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G329" s="2" t="inlineStr">
+        <is>
+          <t>665 Juncal</t>
+        </is>
+      </c>
+      <c r="H329" s="2" t="inlineStr">
+        <is>
+          <t>B1640</t>
+        </is>
+      </c>
+      <c r="I329" s="2" t="inlineStr">
+        <is>
+          <t>https://segundacopa.com.ar</t>
+        </is>
+      </c>
+      <c r="J329" s="2" t="inlineStr"/>
+      <c r="K329" s="2" t="inlineStr"/>
+      <c r="L329" s="2" t="inlineStr"/>
+      <c r="M329" s="2" t="inlineStr"/>
+      <c r="N329" s="2" t="inlineStr">
+        <is>
+          <t>segundacopamt2@gmail.com</t>
+        </is>
+      </c>
+      <c r="O329" s="2" t="inlineStr"/>
+      <c r="P329" s="2" t="inlineStr"/>
+      <c r="Q329" s="2" t="inlineStr"/>
+      <c r="R329" s="2" t="inlineStr"/>
+      <c r="S329" s="2" t="inlineStr">
+        <is>
+          <t>https://es-la.facebook.com/segunda-copa-228461497328200/</t>
+        </is>
+      </c>
+      <c r="T329" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/segunda_copa/</t>
+        </is>
+      </c>
+      <c r="U329" s="2" t="inlineStr"/>
+      <c r="V329" s="2" t="inlineStr"/>
+      <c r="W329" s="2" t="inlineStr">
+        <is>
+          <t>Mariano Toscano</t>
+        </is>
+      </c>
+      <c r="X329" s="2" t="inlineStr">
+        <is>
+          <t>Sales Manager - Sommelier</t>
+        </is>
+      </c>
+      <c r="Y329" s="2" t="inlineStr"/>
+      <c r="Z329" s="2" t="inlineStr"/>
+      <c r="AA329" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/mariano-toscano-a6826a65/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BWI sync — 2026-08-03 12:24 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Argentina.xlsx
+++ b/BWI/bestwine_output/bestwine_Argentina.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA329"/>
+  <dimension ref="A1:AA332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -32250,6 +32250,333 @@
         </is>
       </c>
     </row>
+    <row r="330">
+      <c r="A330" s="2" t="inlineStr">
+        <is>
+          <t>Maycar S.a.</t>
+        </is>
+      </c>
+      <c r="B330" s="2" t="inlineStr">
+        <is>
+          <t>Maycar S.a.</t>
+        </is>
+      </c>
+      <c r="C330" s="2" t="inlineStr">
+        <is>
+          <t>100900</t>
+        </is>
+      </c>
+      <c r="D330" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E330" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F330" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous City of Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G330" s="2" t="inlineStr">
+        <is>
+          <t>1002 Avenida Chorroarín</t>
+        </is>
+      </c>
+      <c r="H330" s="2" t="inlineStr">
+        <is>
+          <t>C1427</t>
+        </is>
+      </c>
+      <c r="I330" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vital.com.ar</t>
+        </is>
+      </c>
+      <c r="J330" s="2" t="inlineStr"/>
+      <c r="K330" s="2" t="inlineStr"/>
+      <c r="L330" s="2" t="inlineStr">
+        <is>
+          <t>1600</t>
+        </is>
+      </c>
+      <c r="M330" s="2" t="inlineStr"/>
+      <c r="N330" s="2" t="inlineStr">
+        <is>
+          <t>info@vital.com.ar</t>
+        </is>
+      </c>
+      <c r="O330" s="2" t="inlineStr"/>
+      <c r="P330" s="2" t="inlineStr">
+        <is>
+          <t>1980</t>
+        </is>
+      </c>
+      <c r="Q330" s="2" t="inlineStr">
+        <is>
+          <t>30-61286533-3</t>
+        </is>
+      </c>
+      <c r="R330" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/vitalsupermayorista/</t>
+        </is>
+      </c>
+      <c r="S330" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/VitalSuperMayorista/</t>
+        </is>
+      </c>
+      <c r="T330" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/vitalsupermayorista/</t>
+        </is>
+      </c>
+      <c r="U330" s="2" t="inlineStr"/>
+      <c r="V330" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/channel/UCyUjBFQz62C-QOSNhlaj-Ww</t>
+        </is>
+      </c>
+      <c r="W330" s="2" t="inlineStr">
+        <is>
+          <t>Agustin Touceda</t>
+        </is>
+      </c>
+      <c r="X330" s="2" t="inlineStr">
+        <is>
+          <t>Buyer</t>
+        </is>
+      </c>
+      <c r="Y330" s="2" t="inlineStr"/>
+      <c r="Z330" s="2" t="inlineStr"/>
+      <c r="AA330" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/agustin-g-touceda/</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="2" t="inlineStr">
+        <is>
+          <t>Maycar S.a.</t>
+        </is>
+      </c>
+      <c r="B331" s="2" t="inlineStr">
+        <is>
+          <t>Maycar S.a.</t>
+        </is>
+      </c>
+      <c r="C331" s="2" t="inlineStr">
+        <is>
+          <t>100900</t>
+        </is>
+      </c>
+      <c r="D331" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E331" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F331" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous City of Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G331" s="2" t="inlineStr">
+        <is>
+          <t>1002 Avenida Chorroarín</t>
+        </is>
+      </c>
+      <c r="H331" s="2" t="inlineStr">
+        <is>
+          <t>C1427</t>
+        </is>
+      </c>
+      <c r="I331" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vital.com.ar</t>
+        </is>
+      </c>
+      <c r="J331" s="2" t="inlineStr"/>
+      <c r="K331" s="2" t="inlineStr"/>
+      <c r="L331" s="2" t="inlineStr">
+        <is>
+          <t>1600</t>
+        </is>
+      </c>
+      <c r="M331" s="2" t="inlineStr"/>
+      <c r="N331" s="2" t="inlineStr">
+        <is>
+          <t>info@vital.com.ar</t>
+        </is>
+      </c>
+      <c r="O331" s="2" t="inlineStr"/>
+      <c r="P331" s="2" t="inlineStr">
+        <is>
+          <t>1980</t>
+        </is>
+      </c>
+      <c r="Q331" s="2" t="inlineStr">
+        <is>
+          <t>30-61286533-3</t>
+        </is>
+      </c>
+      <c r="R331" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/vitalsupermayorista/</t>
+        </is>
+      </c>
+      <c r="S331" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/VitalSuperMayorista/</t>
+        </is>
+      </c>
+      <c r="T331" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/vitalsupermayorista/</t>
+        </is>
+      </c>
+      <c r="U331" s="2" t="inlineStr"/>
+      <c r="V331" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/channel/UCyUjBFQz62C-QOSNhlaj-Ww</t>
+        </is>
+      </c>
+      <c r="W331" s="2" t="inlineStr">
+        <is>
+          <t>Rodrigo Javier</t>
+        </is>
+      </c>
+      <c r="X331" s="2" t="inlineStr">
+        <is>
+          <t>Director Of Operations</t>
+        </is>
+      </c>
+      <c r="Y331" s="2" t="inlineStr"/>
+      <c r="Z331" s="2" t="inlineStr"/>
+      <c r="AA331" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/rodrigo-javier-olivera-28587073/</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="inlineStr">
+        <is>
+          <t>Maycar S.a.</t>
+        </is>
+      </c>
+      <c r="B332" s="2" t="inlineStr">
+        <is>
+          <t>Maycar S.a.</t>
+        </is>
+      </c>
+      <c r="C332" s="2" t="inlineStr">
+        <is>
+          <t>100900</t>
+        </is>
+      </c>
+      <c r="D332" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E332" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F332" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous City of Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G332" s="2" t="inlineStr">
+        <is>
+          <t>1002 Avenida Chorroarín</t>
+        </is>
+      </c>
+      <c r="H332" s="2" t="inlineStr">
+        <is>
+          <t>C1427</t>
+        </is>
+      </c>
+      <c r="I332" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vital.com.ar</t>
+        </is>
+      </c>
+      <c r="J332" s="2" t="inlineStr"/>
+      <c r="K332" s="2" t="inlineStr"/>
+      <c r="L332" s="2" t="inlineStr">
+        <is>
+          <t>1600</t>
+        </is>
+      </c>
+      <c r="M332" s="2" t="inlineStr"/>
+      <c r="N332" s="2" t="inlineStr">
+        <is>
+          <t>info@vital.com.ar</t>
+        </is>
+      </c>
+      <c r="O332" s="2" t="inlineStr"/>
+      <c r="P332" s="2" t="inlineStr">
+        <is>
+          <t>1980</t>
+        </is>
+      </c>
+      <c r="Q332" s="2" t="inlineStr">
+        <is>
+          <t>30-61286533-3</t>
+        </is>
+      </c>
+      <c r="R332" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/vitalsupermayorista/</t>
+        </is>
+      </c>
+      <c r="S332" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/VitalSuperMayorista/</t>
+        </is>
+      </c>
+      <c r="T332" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/vitalsupermayorista/</t>
+        </is>
+      </c>
+      <c r="U332" s="2" t="inlineStr"/>
+      <c r="V332" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/channel/UCyUjBFQz62C-QOSNhlaj-Ww</t>
+        </is>
+      </c>
+      <c r="W332" s="2" t="inlineStr">
+        <is>
+          <t>Ruben Bernel</t>
+        </is>
+      </c>
+      <c r="X332" s="2" t="inlineStr">
+        <is>
+          <t>Regional Operations Manager</t>
+        </is>
+      </c>
+      <c r="Y332" s="2" t="inlineStr"/>
+      <c r="Z332" s="2" t="inlineStr"/>
+      <c r="AA332" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ruben-bernel-17ab82236/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BWI sync — 2026-08-10 10:20 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Argentina.xlsx
+++ b/BWI/bestwine_output/bestwine_Argentina.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA332"/>
+  <dimension ref="A1:AA333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -32577,6 +32577,87 @@
         </is>
       </c>
     </row>
+    <row r="333">
+      <c r="A333" s="2" t="inlineStr">
+        <is>
+          <t>Pietra Distribuidora</t>
+        </is>
+      </c>
+      <c r="B333" s="2" t="inlineStr">
+        <is>
+          <t>Pietra Distribuidora</t>
+        </is>
+      </c>
+      <c r="C333" s="2" t="inlineStr">
+        <is>
+          <t>100688</t>
+        </is>
+      </c>
+      <c r="D333" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E333" s="2" t="inlineStr">
+        <is>
+          <t>Berisso</t>
+        </is>
+      </c>
+      <c r="F333" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G333" s="2" t="inlineStr">
+        <is>
+          <t>250 Calle 34</t>
+        </is>
+      </c>
+      <c r="H333" s="2" t="inlineStr">
+        <is>
+          <t>B1914</t>
+        </is>
+      </c>
+      <c r="I333" s="2" t="inlineStr">
+        <is>
+          <t>https://www.distribuidorapietra.com.ar</t>
+        </is>
+      </c>
+      <c r="J333" s="2" t="inlineStr"/>
+      <c r="K333" s="2" t="inlineStr"/>
+      <c r="L333" s="2" t="inlineStr"/>
+      <c r="M333" s="2" t="inlineStr"/>
+      <c r="N333" s="2" t="inlineStr">
+        <is>
+          <t>info@distribuidorapietra.com.ar</t>
+        </is>
+      </c>
+      <c r="O333" s="2" t="inlineStr">
+        <is>
+          <t>+54 221 666-5674</t>
+        </is>
+      </c>
+      <c r="P333" s="2" t="inlineStr"/>
+      <c r="Q333" s="2" t="inlineStr"/>
+      <c r="R333" s="2" t="inlineStr"/>
+      <c r="S333" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/distribuidorapietra/</t>
+        </is>
+      </c>
+      <c r="T333" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/distribuidorapietra/</t>
+        </is>
+      </c>
+      <c r="U333" s="2" t="inlineStr"/>
+      <c r="V333" s="2" t="inlineStr"/>
+      <c r="W333" s="2" t="inlineStr"/>
+      <c r="X333" s="2" t="inlineStr"/>
+      <c r="Y333" s="2" t="inlineStr"/>
+      <c r="Z333" s="2" t="inlineStr"/>
+      <c r="AA333" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BWI sync — 2026-08-17 09:46 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Argentina.xlsx
+++ b/BWI/bestwine_output/bestwine_Argentina.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA333"/>
+  <dimension ref="A1:AA334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -32658,6 +32658,87 @@
       <c r="Z333" s="2" t="inlineStr"/>
       <c r="AA333" s="2" t="inlineStr"/>
     </row>
+    <row r="334">
+      <c r="A334" s="2" t="inlineStr">
+        <is>
+          <t>Pietra Distribuidora</t>
+        </is>
+      </c>
+      <c r="B334" s="2" t="inlineStr">
+        <is>
+          <t>Pietra Distribuidora</t>
+        </is>
+      </c>
+      <c r="C334" s="2" t="inlineStr">
+        <is>
+          <t>100688</t>
+        </is>
+      </c>
+      <c r="D334" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E334" s="2" t="inlineStr">
+        <is>
+          <t>Berisso</t>
+        </is>
+      </c>
+      <c r="F334" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G334" s="2" t="inlineStr">
+        <is>
+          <t>250 Calle 34</t>
+        </is>
+      </c>
+      <c r="H334" s="2" t="inlineStr">
+        <is>
+          <t>B1914</t>
+        </is>
+      </c>
+      <c r="I334" s="2" t="inlineStr">
+        <is>
+          <t>https://www.distribuidorapietra.com.ar</t>
+        </is>
+      </c>
+      <c r="J334" s="2" t="inlineStr"/>
+      <c r="K334" s="2" t="inlineStr"/>
+      <c r="L334" s="2" t="inlineStr"/>
+      <c r="M334" s="2" t="inlineStr"/>
+      <c r="N334" s="2" t="inlineStr">
+        <is>
+          <t>info@distribuidorapietra.com.ar</t>
+        </is>
+      </c>
+      <c r="O334" s="2" t="inlineStr">
+        <is>
+          <t>+54 221 666-5674</t>
+        </is>
+      </c>
+      <c r="P334" s="2" t="inlineStr"/>
+      <c r="Q334" s="2" t="inlineStr"/>
+      <c r="R334" s="2" t="inlineStr"/>
+      <c r="S334" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/distribuidorapietra/</t>
+        </is>
+      </c>
+      <c r="T334" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/distribuidorapietra/</t>
+        </is>
+      </c>
+      <c r="U334" s="2" t="inlineStr"/>
+      <c r="V334" s="2" t="inlineStr"/>
+      <c r="W334" s="2" t="inlineStr"/>
+      <c r="X334" s="2" t="inlineStr"/>
+      <c r="Y334" s="2" t="inlineStr"/>
+      <c r="Z334" s="2" t="inlineStr"/>
+      <c r="AA334" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BWI sync — 2026-08-24 09:52 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Argentina.xlsx
+++ b/BWI/bestwine_output/bestwine_Argentina.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA334"/>
+  <dimension ref="A1:AA335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -32739,6 +32739,87 @@
       <c r="Z334" s="2" t="inlineStr"/>
       <c r="AA334" s="2" t="inlineStr"/>
     </row>
+    <row r="335">
+      <c r="A335" s="2" t="inlineStr">
+        <is>
+          <t>Pietra Distribuidora</t>
+        </is>
+      </c>
+      <c r="B335" s="2" t="inlineStr">
+        <is>
+          <t>Pietra Distribuidora</t>
+        </is>
+      </c>
+      <c r="C335" s="2" t="inlineStr">
+        <is>
+          <t>100688</t>
+        </is>
+      </c>
+      <c r="D335" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E335" s="2" t="inlineStr">
+        <is>
+          <t>Berisso</t>
+        </is>
+      </c>
+      <c r="F335" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G335" s="2" t="inlineStr">
+        <is>
+          <t>250 Calle 34</t>
+        </is>
+      </c>
+      <c r="H335" s="2" t="inlineStr">
+        <is>
+          <t>B1914</t>
+        </is>
+      </c>
+      <c r="I335" s="2" t="inlineStr">
+        <is>
+          <t>https://www.distribuidorapietra.com.ar</t>
+        </is>
+      </c>
+      <c r="J335" s="2" t="inlineStr"/>
+      <c r="K335" s="2" t="inlineStr"/>
+      <c r="L335" s="2" t="inlineStr"/>
+      <c r="M335" s="2" t="inlineStr"/>
+      <c r="N335" s="2" t="inlineStr">
+        <is>
+          <t>info@distribuidorapietra.com.ar</t>
+        </is>
+      </c>
+      <c r="O335" s="2" t="inlineStr">
+        <is>
+          <t>+54 221 666-5674</t>
+        </is>
+      </c>
+      <c r="P335" s="2" t="inlineStr"/>
+      <c r="Q335" s="2" t="inlineStr"/>
+      <c r="R335" s="2" t="inlineStr"/>
+      <c r="S335" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/distribuidorapietra/</t>
+        </is>
+      </c>
+      <c r="T335" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/distribuidorapietra/</t>
+        </is>
+      </c>
+      <c r="U335" s="2" t="inlineStr"/>
+      <c r="V335" s="2" t="inlineStr"/>
+      <c r="W335" s="2" t="inlineStr"/>
+      <c r="X335" s="2" t="inlineStr"/>
+      <c r="Y335" s="2" t="inlineStr"/>
+      <c r="Z335" s="2" t="inlineStr"/>
+      <c r="AA335" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BWI sync — 2026-08-31 16:51 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Argentina.xlsx
+++ b/BWI/bestwine_output/bestwine_Argentina.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA335"/>
+  <dimension ref="A1:AA336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -32820,6 +32820,87 @@
       <c r="Z335" s="2" t="inlineStr"/>
       <c r="AA335" s="2" t="inlineStr"/>
     </row>
+    <row r="336">
+      <c r="A336" s="2" t="inlineStr">
+        <is>
+          <t>Pietra Distribuidora</t>
+        </is>
+      </c>
+      <c r="B336" s="2" t="inlineStr">
+        <is>
+          <t>Pietra Distribuidora</t>
+        </is>
+      </c>
+      <c r="C336" s="2" t="inlineStr">
+        <is>
+          <t>100688</t>
+        </is>
+      </c>
+      <c r="D336" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E336" s="2" t="inlineStr">
+        <is>
+          <t>Berisso</t>
+        </is>
+      </c>
+      <c r="F336" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G336" s="2" t="inlineStr">
+        <is>
+          <t>250 Calle 34</t>
+        </is>
+      </c>
+      <c r="H336" s="2" t="inlineStr">
+        <is>
+          <t>B1914</t>
+        </is>
+      </c>
+      <c r="I336" s="2" t="inlineStr">
+        <is>
+          <t>https://www.distribuidorapietra.com.ar</t>
+        </is>
+      </c>
+      <c r="J336" s="2" t="inlineStr"/>
+      <c r="K336" s="2" t="inlineStr"/>
+      <c r="L336" s="2" t="inlineStr"/>
+      <c r="M336" s="2" t="inlineStr"/>
+      <c r="N336" s="2" t="inlineStr">
+        <is>
+          <t>info@distribuidorapietra.com.ar</t>
+        </is>
+      </c>
+      <c r="O336" s="2" t="inlineStr">
+        <is>
+          <t>+54 221 666-5674</t>
+        </is>
+      </c>
+      <c r="P336" s="2" t="inlineStr"/>
+      <c r="Q336" s="2" t="inlineStr"/>
+      <c r="R336" s="2" t="inlineStr"/>
+      <c r="S336" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/distribuidorapietra/</t>
+        </is>
+      </c>
+      <c r="T336" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/distribuidorapietra/</t>
+        </is>
+      </c>
+      <c r="U336" s="2" t="inlineStr"/>
+      <c r="V336" s="2" t="inlineStr"/>
+      <c r="W336" s="2" t="inlineStr"/>
+      <c r="X336" s="2" t="inlineStr"/>
+      <c r="Y336" s="2" t="inlineStr"/>
+      <c r="Z336" s="2" t="inlineStr"/>
+      <c r="AA336" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BWI sync — 2026-09-07 14:55 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Argentina.xlsx
+++ b/BWI/bestwine_output/bestwine_Argentina.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA336"/>
+  <dimension ref="A1:AA337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -32901,6 +32901,87 @@
       <c r="Z336" s="2" t="inlineStr"/>
       <c r="AA336" s="2" t="inlineStr"/>
     </row>
+    <row r="337">
+      <c r="A337" s="2" t="inlineStr">
+        <is>
+          <t>Pietra Distribuidora</t>
+        </is>
+      </c>
+      <c r="B337" s="2" t="inlineStr">
+        <is>
+          <t>Pietra Distribuidora</t>
+        </is>
+      </c>
+      <c r="C337" s="2" t="inlineStr">
+        <is>
+          <t>100688</t>
+        </is>
+      </c>
+      <c r="D337" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E337" s="2" t="inlineStr">
+        <is>
+          <t>Berisso</t>
+        </is>
+      </c>
+      <c r="F337" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G337" s="2" t="inlineStr">
+        <is>
+          <t>250 Calle 34</t>
+        </is>
+      </c>
+      <c r="H337" s="2" t="inlineStr">
+        <is>
+          <t>B1914</t>
+        </is>
+      </c>
+      <c r="I337" s="2" t="inlineStr">
+        <is>
+          <t>https://www.distribuidorapietra.com.ar</t>
+        </is>
+      </c>
+      <c r="J337" s="2" t="inlineStr"/>
+      <c r="K337" s="2" t="inlineStr"/>
+      <c r="L337" s="2" t="inlineStr"/>
+      <c r="M337" s="2" t="inlineStr"/>
+      <c r="N337" s="2" t="inlineStr">
+        <is>
+          <t>info@distribuidorapietra.com.ar</t>
+        </is>
+      </c>
+      <c r="O337" s="2" t="inlineStr">
+        <is>
+          <t>+54 221 666-5674</t>
+        </is>
+      </c>
+      <c r="P337" s="2" t="inlineStr"/>
+      <c r="Q337" s="2" t="inlineStr"/>
+      <c r="R337" s="2" t="inlineStr"/>
+      <c r="S337" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/distribuidorapietra/</t>
+        </is>
+      </c>
+      <c r="T337" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/distribuidorapietra/</t>
+        </is>
+      </c>
+      <c r="U337" s="2" t="inlineStr"/>
+      <c r="V337" s="2" t="inlineStr"/>
+      <c r="W337" s="2" t="inlineStr"/>
+      <c r="X337" s="2" t="inlineStr"/>
+      <c r="Y337" s="2" t="inlineStr"/>
+      <c r="Z337" s="2" t="inlineStr"/>
+      <c r="AA337" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>